<commit_message>
User stories for MVP added
</commit_message>
<xml_diff>
--- a/Docs/ProductBacklog.xlsx
+++ b/Docs/ProductBacklog.xlsx
@@ -5,11 +5,11 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Sheet3" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Initial Draft" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="MVP" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Feature Dump" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="171">
   <si>
     <t xml:space="preserve">Phase</t>
   </si>
@@ -154,6 +154,382 @@
   </si>
   <si>
     <t xml:space="preserve">Selecting songs as per beginning, Middle &amp; Climax of a show</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User Stories</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Google auth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sign-in/sign-up with Google</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a new user, I want to sign up with Google OAuth so that I can quickly create an account without a password
+As an existing user, I want to log in with Google so that I don't have to remember separate credentials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name, Sex, Age, Nationality</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Predicts listening patterns &amp; tastes from identity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want to provide my basic demographics so that RedDust can personalize recommendations based on my profile
+As a user, I want to update my profile information so that recommendations stay accurate over time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Music preferences, past choices</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Understands music preferences from the user himself</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want to share my past favorite songs so that RedDust understands my music taste
+As a user, I want RedDust to learn from my listening history so that recommendations improve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Daily Check-in &amp; Mood Detection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Daily Check-in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User logs in daily and shares mood via voice/text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want to check in daily and share my mood so that RedDust understands my current emotional state
+As a user, I want to quickly log my mood in under 30 seconds so that I'm encouraged to check in daily</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mood Detection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI detects emotional state from conversation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As RedDust, I want to analyze user's voice/text to detect their emotional state so that I can provide appropriate recommendations
+As a user, I want RedDust to understand nuanced emotions from my words so that it doesn't oversimplify my feelings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voice Commands</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User can speak instead of typing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want to speak my mood instead of typing so that I can interact hands-free while busy
+As a user, I want voice commands to work in background so that I can use RedDust while driving or exercising</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Life Situation Understanding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Context Capture</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI understands user context (exams, work, relationships)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want to tell RedDust about my life context (exams, work stress, relationships) so that it understands why I feel a certain way
+As RedDust, I want to remember user's context from past conversations so that recommendations stay relevant to their situation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voice-enabled Prompts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voice interface for situation input</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want to provide context information via voice so that I can share details hands-free
+As RedDust, I want to prompt users with smart follow-up questions using voice so that I can gather context conversationally</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Playlist Generation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User mood + situation + duration → personalized playlist</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want RedDust to generate a playlist based on my mood and life situation so that I get personalized recommendations
+As a user, I want to specify playlist duration so that I get exactly the right amount of music for my activity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Energy Curve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Playlist structured by mood intensity from trends captured</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want my playlist to have a structured energy flow (starting calm and building up, or vice versa) so that it matches my needs
+As RedDust, I want to sequence songs by energy intensity based on the user's mood trajectory so that the listening experience is cohesive</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Language &amp; Age-appropriate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Songs match user preference and age</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want songs to match my language preferences so that I can understand and connect with lyrics
+As a parent/user, I want RedDust to filter age-appropriate songs so that young users only hear suitable content</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Music Playback</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YouTube Music Integration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Play songs from AI-generated playlists</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want to play songs from RedDust's recommended playlists via YouTube Music so that I can listen to high-quality audio
+As RedDust, I want to search and retrieve songs from YouTube Music so that users have access to a vast music library</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Play/Pause Controls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Basic playback controls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want basic playback controls so that I can pause when interrupted and resume later
+As a user, I want to control playback from RedDust's interface so that I don't have to switch between apps</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skip &amp; Like</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skip to next song or like/dislike track (these happen in RedDust, not music streaming app)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want to skip songs I don't like so that I only hear music that resonates with me
+As a user, I want to like/dislike songs so that RedDust learns what I enjoy and improves future recommendations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Personal Memory System</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Favorite Songs &amp; Artists</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Store user favorite songs and artists</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want to save favorite songs in a library so that I can revisit them later
+As a user, I want to maintain a list of favorite artists so that RedDust knows which creators I love</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mood Patterns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Track which songs user listens to in different moods</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As RedDust, I want to track which songs the user listens to in different moods so that I can predict what works for them
+As a user, I want to see which songs I play when I'm happy/sad/focused so that I understand my own patterns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conversation History</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Store and recall past conversations for personalization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As RedDust, I want to store past conversations so that I can reference them and provide personalized context
+As a user, I want RedDust to remember what I told it previously so that I don't have to repeat myself</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Listening Preferences</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remember language and genre preferences</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As RedDust, I want to remember user's language and genre preferences so that future recommendations are aligned
+As a user, I want my preferences to persist so that RedDust stays tuned to my tastes over time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recommendation Engine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Learn from Skips</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Negative signal: skip indicates dislike</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As RedDust, I want to register when a user skips a song so that I know it didn't match their taste
+As a user, I want skips to negatively impact future recommendations so that RedDust learns what NOT to recommend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Learn from Likes &amp; Replays</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Positive signals improve recommendations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As RedDust, I want to track when users replay songs so that I know those are strong preferences
+As a user, I want RedDust to boost recommendations of songs I like and replay frequently</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Time-of-day Learning</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Different songs recommended based on time of day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As RedDust, I want to notice patterns in what users listen to at different times so that I can recommend appropriately
+As a user, I want different recommendations in the morning vs evening so that songs match my daily rhythm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mood-based Learning</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recommendations adapt based on mood patterns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As RedDust, I want to adapt recommendations based on recurring mood patterns so that I anticipate user needs
+As a user, I want RedDust to know that when I'm stressed, I like lo-fi beats, not heavy metal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Well-being Dashboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mood Trend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visualize mood over time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want to see a visual graph of my mood over time so that I understand my emotional patterns
+As a user, I want to identify what improves or worsens my mood by looking at trends over weeks/months</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stress Trend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Track stress levels</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want to track stress levels so that I can see if RedDust's music helps reduce stress
+As a user, I want to correlate stress spikes with events so that I understand my stress triggers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Energy Trend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monitor energy patterns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want to monitor my energy levels over time so that I can plan activities accordingly
+As RedDust, I want to suggest more energizing music when I detect low energy patterns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Energy/mental state curve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Captures moods/mental energy throughout the day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want to see how my mental energy fluctuates throughout the day so that I can schedule tasks better
+As RedDust, I want to recommend music that matches the user's energy curve to keep them productive</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Listening Pattern</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Show listening habits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want to see my listening habits displayed so that I can understand my music consumption
+As RedDust, I want to analyze listening patterns to recommend at the right moment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Listening Hours</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Display total hours user listened</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want to see total hours I've listened so that I can appreciate my music engagement
+As a user, I want to track listening time by mood/genre so that I understand where I spend the most time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Artist/Genre/Song Facts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Song Information Display</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1-2 line fact about artist/genre/song on selection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want to see facts about the artist/genre/song when I select it so that I learn while I listen
+As a user, I want interesting context about songs so that my listening experience is educational and engaging</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto-generated Facts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Facts generated for all songs in prescription playlist</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As RedDust, I want to generate interesting facts for every song in the playlist so that users always have context
+As a user, I want AI-generated facts about songs so that the conversation between songs is enriching</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Song lyrics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Show the lyrics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want to read lyrics while listening so that I can understand what the song means
+As a user, I want to sing along with accurate, real-time lyrics displayed on my screen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Song Recognition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voice-enabled Recording</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User taps button to record song snippet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want to record a snippet of a song by tapping a button so that I can identify unknown songs
+As a user, I want to capture music I hear in the background so that I can add it to my library</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Song Identification</t>
+  </si>
+  <si>
+    <t xml:space="preserve">App identifies song from audio (Shazam-like)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As RedDust, I want to identify songs from audio samples so that users can discover and save new music
+As a user, I want instant identification of songs I hear so that I never lose track of music I like</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add to Library</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Option to add identified song to favorites</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want to add identified songs to my favorites so that I don't forget about them
+As a user, I want to build my music library by saving discovered songs</t>
   </si>
   <si>
     <t xml:space="preserve">Extra</t>
@@ -202,7 +578,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -233,6 +609,13 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -242,10 +625,73 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin"/>
       <top/>
       <bottom/>
       <diagonal/>
@@ -276,29 +722,89 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -494,7 +1000,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G29"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.58984375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.63"/>
@@ -506,7 +1012,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="2" width="10.16"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="30.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -525,7 +1031,7 @@
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
         <v>5</v>
       </c>
@@ -539,7 +1045,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5"/>
       <c r="B3" s="1" t="n">
         <v>3</v>
@@ -551,55 +1057,47 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5"/>
       <c r="B4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>8</v>
-      </c>
+      <c r="C4" s="5"/>
       <c r="D4" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5"/>
       <c r="B5" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>8</v>
-      </c>
+      <c r="C5" s="5"/>
       <c r="D5" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5"/>
       <c r="B6" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>8</v>
-      </c>
+      <c r="C6" s="5"/>
       <c r="D6" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5"/>
       <c r="B7" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>8</v>
-      </c>
+      <c r="C7" s="5"/>
       <c r="D7" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5"/>
       <c r="C8" s="2" t="s">
         <v>14</v>
@@ -608,7 +1106,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5"/>
       <c r="B9" s="1" t="n">
         <v>3</v>
@@ -620,7 +1118,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5"/>
       <c r="B10" s="1" t="n">
         <v>3</v>
@@ -632,7 +1130,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5"/>
       <c r="B11" s="1" t="n">
         <v>3</v>
@@ -644,7 +1142,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5"/>
       <c r="B12" s="1" t="n">
         <v>3</v>
@@ -656,7 +1154,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5"/>
       <c r="B13" s="1" t="n">
         <v>3</v>
@@ -668,7 +1166,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5"/>
       <c r="B14" s="1" t="n">
         <v>3</v>
@@ -680,7 +1178,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5"/>
       <c r="B15" s="1" t="n">
         <v>3</v>
@@ -692,7 +1190,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5"/>
       <c r="B16" s="1" t="n">
         <v>3</v>
@@ -702,7 +1200,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="5"/>
       <c r="B17" s="1" t="n">
         <v>3</v>
@@ -712,7 +1210,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="5"/>
       <c r="B18" s="1" t="n">
         <v>3</v>
@@ -722,7 +1220,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="5"/>
       <c r="B19" s="1" t="n">
         <v>3</v>
@@ -734,7 +1232,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="5"/>
       <c r="B20" s="1" t="n">
         <v>3</v>
@@ -746,7 +1244,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5"/>
       <c r="B21" s="1" t="n">
         <v>3</v>
@@ -758,7 +1256,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="5"/>
       <c r="B22" s="1" t="n">
         <v>3</v>
@@ -770,7 +1268,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="5"/>
       <c r="B23" s="1" t="n">
         <v>3</v>
@@ -782,7 +1280,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
         <v>35</v>
       </c>
@@ -796,7 +1294,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C25" s="2" t="s">
         <v>36</v>
       </c>
@@ -804,7 +1302,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C26" s="2" t="s">
         <v>36</v>
       </c>
@@ -812,7 +1310,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C27" s="2" t="s">
         <v>36</v>
       </c>
@@ -820,7 +1318,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C28" s="2" t="s">
         <v>36</v>
       </c>
@@ -828,7 +1326,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C29" s="2" t="s">
         <v>42</v>
       </c>
@@ -857,126 +1355,625 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F35"/>
+  <sheetFormatPr defaultColWidth="60.00390625" defaultRowHeight="13.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12.58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="51.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="66.52"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="1" width="60"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="60.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
+    <row r="1" s="3" customFormat="true" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5"/>
-      <c r="C3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B3" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5"/>
-      <c r="C4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="9"/>
+      <c r="D4" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="E4" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="F4" s="15" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5"/>
-    </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5"/>
-    </row>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" s="9"/>
+      <c r="D6" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="E6" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="F6" s="18" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5"/>
-    </row>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" s="9"/>
+      <c r="D7" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="F7" s="15" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5"/>
-    </row>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F8" s="13" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5"/>
-    </row>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" s="9"/>
+      <c r="D9" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="F9" s="15" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5"/>
-    </row>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5"/>
-    </row>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" s="9"/>
+      <c r="D11" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="F11" s="18" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5"/>
-    </row>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C12" s="9"/>
+      <c r="D12" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="E12" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="F12" s="15" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5"/>
-    </row>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5"/>
-    </row>
-    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" s="9"/>
+      <c r="D14" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="E14" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="F14" s="18" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5"/>
-    </row>
-    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" s="9"/>
+      <c r="D15" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="E15" s="19" t="s">
+        <v>91</v>
+      </c>
+      <c r="F15" s="15" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5"/>
-    </row>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="F16" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5"/>
-    </row>
-    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" s="9"/>
+      <c r="D17" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="E17" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="F17" s="18" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5"/>
-    </row>
-    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" s="9"/>
+      <c r="D18" s="16" t="s">
+        <v>100</v>
+      </c>
+      <c r="E18" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="F18" s="18" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5"/>
-    </row>
-    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" s="9"/>
+      <c r="D19" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="E19" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="F19" s="15" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5"/>
-    </row>
-    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="F20" s="13" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5"/>
-    </row>
-    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C21" s="9"/>
+      <c r="D21" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="E21" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="F21" s="18" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5"/>
-    </row>
-    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C22" s="9"/>
+      <c r="D22" s="16" t="s">
+        <v>113</v>
+      </c>
+      <c r="E22" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="F22" s="18" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5"/>
+      <c r="B23" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C23" s="9"/>
+      <c r="D23" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="E23" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="F23" s="15" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5"/>
+      <c r="B24" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="D24" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="E24" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="F24" s="13" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="5"/>
+      <c r="B25" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" s="9"/>
+      <c r="D25" s="16" t="s">
+        <v>123</v>
+      </c>
+      <c r="E25" s="17" t="s">
+        <v>124</v>
+      </c>
+      <c r="F25" s="18" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="5"/>
+      <c r="B26" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C26" s="9"/>
+      <c r="D26" s="16" t="s">
+        <v>126</v>
+      </c>
+      <c r="E26" s="17" t="s">
+        <v>127</v>
+      </c>
+      <c r="F26" s="18" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="5"/>
+      <c r="B27" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C27" s="9"/>
+      <c r="D27" s="16" t="s">
+        <v>129</v>
+      </c>
+      <c r="E27" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="F27" s="18" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="5"/>
+      <c r="B28" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C28" s="9"/>
+      <c r="D28" s="16" t="s">
+        <v>132</v>
+      </c>
+      <c r="E28" s="17" t="s">
+        <v>133</v>
+      </c>
+      <c r="F28" s="18" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="5"/>
+      <c r="B29" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C29" s="9"/>
+      <c r="D29" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="E29" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="F29" s="15" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="5"/>
+      <c r="B30" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C30" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>139</v>
+      </c>
+      <c r="E30" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="F30" s="13" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="5"/>
+      <c r="B31" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C31" s="9"/>
+      <c r="D31" s="16" t="s">
+        <v>142</v>
+      </c>
+      <c r="E31" s="17" t="s">
+        <v>143</v>
+      </c>
+      <c r="F31" s="18" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="5"/>
+      <c r="B32" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C32" s="9"/>
+      <c r="D32" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="E32" s="14" t="s">
+        <v>146</v>
+      </c>
+      <c r="F32" s="15" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="5"/>
+      <c r="B33" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C33" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="D33" s="12" t="s">
+        <v>149</v>
+      </c>
+      <c r="E33" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="F33" s="13" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="5"/>
+      <c r="B34" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C34" s="9"/>
+      <c r="D34" s="16" t="s">
+        <v>152</v>
+      </c>
+      <c r="E34" s="17" t="s">
+        <v>153</v>
+      </c>
+      <c r="F34" s="18" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="60.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="5"/>
+      <c r="B35" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C35" s="9"/>
+      <c r="D35" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="E35" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="F35" s="15" t="s">
+        <v>157</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:A23"/>
+  <mergeCells count="11">
+    <mergeCell ref="A2:A35"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="C5:C7"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="C10:C12"/>
+    <mergeCell ref="C13:C15"/>
+    <mergeCell ref="C16:C19"/>
+    <mergeCell ref="C20:C23"/>
+    <mergeCell ref="C24:C29"/>
+    <mergeCell ref="C30:C32"/>
+    <mergeCell ref="C33:C35"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12 &amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12 &amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -987,74 +1984,74 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:A13"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="73.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="20" width="73.31"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
-        <v>56</v>
+    <row r="1" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="20" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="20" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="20" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="20" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="20" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="20" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="20" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="20" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="20" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="20" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="20" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="20" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="20" t="s">
+        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -1062,8 +2059,8 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12 &amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12 &amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>